<commit_message>
Report update @ 01-Sep-2025 08:48:33
</commit_message>
<xml_diff>
--- a/wildlife/reports/United-Kingdom/abundance/Abingdon/Birds/abundance.xlsx
+++ b/wildlife/reports/United-Kingdom/abundance/Abingdon/Birds/abundance.xlsx
@@ -743,10 +743,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="D20" t="n">
-        <v>1484</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="21">
@@ -1095,10 +1095,10 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="D42" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
     </row>
     <row r="43">
@@ -1287,10 +1287,10 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1464</v>
+        <v>1465</v>
       </c>
       <c r="D54" t="n">
-        <v>1353</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="55">
@@ -1783,10 +1783,10 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3261</v>
+        <v>3262</v>
       </c>
       <c r="D85" t="n">
-        <v>1695</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="86">

</xml_diff>